<commit_message>
Refactor admin portal and enhance Shariah compliance
- Introduced HalalBourse-specific rules for compliance logic.
- Refactored admin portal with lazy-loaded routes and new layout.
- Added endpoints for managing FaisalBank/Ostoul PDF reports.
- Improved Shariah compliance data integrity with audits and fixes.
- Enhanced UI for financial metrics and compliance statuses.
- Added new infrastructure test project and placeholder tests.
- Improved error handling for database update exceptions.
- Refactored background services for long delay handling.
</commit_message>
<xml_diff>
--- a/Sectoral-Indices.xlsx
+++ b/Sectoral-Indices.xlsx
@@ -1,15 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\borsa\Meezan\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBEF0C52-60CA-4F0B-85FA-971495A42E57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="105" yWindow="105" windowWidth="10005" windowHeight="7005"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -2320,8 +2337,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -2373,11 +2390,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2385,13 +2403,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2429,7 +2455,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -2463,6 +2489,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2497,9 +2524,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2672,23 +2700,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:G229"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="60.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="60.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.88671875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2711,7 +2739,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -2730,11 +2758,11 @@
       <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="3">
-        <v>5.2075276618800036E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="G2" s="4">
+        <v>5.2075276618800039</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -2753,11 +2781,11 @@
       <c r="F3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="3">
-        <v>2.9939586697506886E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="G3" s="4">
+        <v>2.9939586697506888</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -2776,11 +2804,11 @@
       <c r="F4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="3">
-        <v>2.2684307888757617E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="G4" s="4">
+        <v>2.2684307888757616</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
@@ -2799,11 +2827,11 @@
       <c r="F5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="3">
-        <v>8.2111217063873341E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="G5" s="4">
+        <v>0.82111217063873343</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -2822,11 +2850,11 @@
       <c r="F6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="3">
-        <v>0.12848513344571966</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="G6" s="4">
+        <v>12.848513344571966</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -2845,11 +2873,11 @@
       <c r="F7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="3">
-        <v>0.35000000000000026</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="G7" s="4">
+        <v>35.000000000000028</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>32</v>
       </c>
@@ -2868,11 +2896,11 @@
       <c r="F8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="3">
-        <v>2.2368431243624285E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+      <c r="G8" s="4">
+        <v>2.2368431243624287</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>36</v>
       </c>
@@ -2891,11 +2919,11 @@
       <c r="F9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="3">
-        <v>3.4409738660153233E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="G9" s="4">
+        <v>3.4409738660153231</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>40</v>
       </c>
@@ -2914,11 +2942,11 @@
       <c r="F10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="3">
-        <v>2.1906442726330043E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="G10" s="4">
+        <v>2.1906442726330044</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>44</v>
       </c>
@@ -2937,11 +2965,11 @@
       <c r="F11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G11" s="3">
-        <v>0.27816898729805134</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+      <c r="G11" s="4">
+        <v>27.816898729805136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>48</v>
       </c>
@@ -2960,11 +2988,11 @@
       <c r="F12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G12" s="3">
-        <v>1.6492361568786647E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="G12" s="4">
+        <v>1.6492361568786646</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>52</v>
       </c>
@@ -2983,38 +3011,40 @@
       <c r="F13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="3">
-        <v>3.5258612145882648E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+      <c r="G13" s="4">
+        <v>3.5258612145882648</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
+      <c r="G14" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
-    </row>
-    <row r="16" spans="1:7">
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>56</v>
       </c>
@@ -3033,11 +3063,11 @@
       <c r="F17" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G17" s="3">
-        <v>1.0931477790667625E-2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="G17" s="4">
+        <v>1.0931477790667625</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>62</v>
       </c>
@@ -3056,11 +3086,11 @@
       <c r="F18" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G18" s="3">
-        <v>1.6915373342775378E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="G18" s="4">
+        <v>1.6915373342775379</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>66</v>
       </c>
@@ -3079,11 +3109,11 @@
       <c r="F19" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G19" s="3">
-        <v>0.11043423374392047</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="G19" s="4">
+        <v>11.043423374392047</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>70</v>
       </c>
@@ -3102,11 +3132,11 @@
       <c r="F20" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G20" s="3">
-        <v>0.30468670596799746</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="G20" s="4">
+        <v>30.468670596799747</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>74</v>
       </c>
@@ -3125,11 +3155,11 @@
       <c r="F21" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G21" s="3">
-        <v>3.1768387940914793E-2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="G21" s="4">
+        <v>3.1768387940914793</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>78</v>
       </c>
@@ -3148,11 +3178,11 @@
       <c r="F22" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G22" s="3">
-        <v>1.9551122426791228E-2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
+      <c r="G22" s="4">
+        <v>1.9551122426791228</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>82</v>
       </c>
@@ -3171,11 +3201,11 @@
       <c r="F23" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G23" s="3">
-        <v>6.1736919795813888E-2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
+      <c r="G23" s="4">
+        <v>6.1736919795813892</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>86</v>
       </c>
@@ -3194,11 +3224,11 @@
       <c r="F24" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G24" s="3">
-        <v>1.1688203730224233E-2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
+      <c r="G24" s="4">
+        <v>1.1688203730224234</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>90</v>
       </c>
@@ -3217,11 +3247,11 @@
       <c r="F25" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G25" s="3">
-        <v>7.2676512082865061E-2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
+      <c r="G25" s="4">
+        <v>7.2676512082865061</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>94</v>
       </c>
@@ -3240,11 +3270,11 @@
       <c r="F26" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G26" s="3">
-        <v>0.1959295401598872</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
+      <c r="G26" s="4">
+        <v>19.59295401598872</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>98</v>
       </c>
@@ -3263,11 +3293,11 @@
       <c r="F27" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G27" s="3">
-        <v>3.2834874704996474E-3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
+      <c r="G27" s="4">
+        <v>0.32834874704996475</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>102</v>
       </c>
@@ -3286,11 +3316,11 @@
       <c r="F28" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G28" s="3">
-        <v>2.2693325259280129E-2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
+      <c r="G28" s="4">
+        <v>2.269332525928013</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>106</v>
       </c>
@@ -3309,38 +3339,40 @@
       <c r="F29" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G29" s="3">
-        <v>0.13770471028836284</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
+      <c r="G29" s="4">
+        <v>13.770471028836283</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
-      <c r="G30" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
+      <c r="G30" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
-    </row>
-    <row r="32" spans="1:7">
+      <c r="G31" s="4"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
-    </row>
-    <row r="33" spans="1:7">
+      <c r="G32" s="4"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>110</v>
       </c>
@@ -3359,11 +3391,11 @@
       <c r="F33" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G33" s="3">
-        <v>6.4540129002803549E-3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
+      <c r="G33" s="4">
+        <v>0.64540129002803548</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>116</v>
       </c>
@@ -3382,11 +3414,11 @@
       <c r="F34" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G34" s="3">
-        <v>1.5501846581234057E-2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
+      <c r="G34" s="4">
+        <v>1.5501846581234058</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>120</v>
       </c>
@@ -3405,11 +3437,11 @@
       <c r="F35" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G35" s="3">
-        <v>0.11774691480718003</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7">
+      <c r="G35" s="4">
+        <v>11.774691480718003</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>124</v>
       </c>
@@ -3428,11 +3460,11 @@
       <c r="F36" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G36" s="3">
-        <v>1.7775528408393304E-2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7">
+      <c r="G36" s="4">
+        <v>1.7775528408393304</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>128</v>
       </c>
@@ -3451,11 +3483,11 @@
       <c r="F37" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G37" s="3">
-        <v>1.0713427205723554E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
+      <c r="G37" s="4">
+        <v>1.0713427205723554</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>132</v>
       </c>
@@ -3474,11 +3506,11 @@
       <c r="F38" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G38" s="3">
-        <v>2.2735688897907821E-2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
+      <c r="G38" s="4">
+        <v>2.273568889790782</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>136</v>
       </c>
@@ -3497,11 +3529,11 @@
       <c r="F39" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G39" s="3">
-        <v>0.16078688302981936</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
+      <c r="G39" s="4">
+        <v>16.078688302981938</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>140</v>
       </c>
@@ -3520,11 +3552,11 @@
       <c r="F40" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G40" s="3">
-        <v>0.2298744551286182</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
+      <c r="G40" s="4">
+        <v>22.987445512861822</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>144</v>
       </c>
@@ -3543,11 +3575,11 @@
       <c r="F41" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G41" s="3">
-        <v>0.26725664258714599</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7">
+      <c r="G41" s="4">
+        <v>26.725664258714598</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>148</v>
       </c>
@@ -3566,38 +3598,40 @@
       <c r="F42" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G42" s="3">
-        <v>0.15115460045369741</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7">
+      <c r="G42" s="4">
+        <v>15.115460045369741</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
-      <c r="G43" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7">
+      <c r="G43" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
-    </row>
-    <row r="45" spans="1:7">
+      <c r="G44" s="4"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
-    </row>
-    <row r="46" spans="1:7">
+      <c r="G45" s="4"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>152</v>
       </c>
@@ -3616,11 +3650,11 @@
       <c r="F46" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G46" s="3">
-        <v>1.7302242779024563E-2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7">
+      <c r="G46" s="4">
+        <v>1.7302242779024564</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>158</v>
       </c>
@@ -3639,11 +3673,11 @@
       <c r="F47" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G47" s="3">
-        <v>1.934742570681456E-2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7">
+      <c r="G47" s="4">
+        <v>1.9347425706814561</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>162</v>
       </c>
@@ -3662,11 +3696,11 @@
       <c r="F48" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G48" s="3">
-        <v>0.20622747805265476</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7">
+      <c r="G48" s="4">
+        <v>20.622747805265476</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>166</v>
       </c>
@@ -3685,11 +3719,11 @@
       <c r="F49" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G49" s="3">
-        <v>5.6862735078696193E-2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7">
+      <c r="G49" s="4">
+        <v>5.6862735078696192</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>170</v>
       </c>
@@ -3708,11 +3742,11 @@
       <c r="F50" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G50" s="3">
-        <v>7.8039926999973822E-2</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7">
+      <c r="G50" s="4">
+        <v>7.8039926999973819</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>174</v>
       </c>
@@ -3731,11 +3765,11 @@
       <c r="F51" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G51" s="3">
-        <v>3.7989027935367681E-2</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7">
+      <c r="G51" s="4">
+        <v>3.7989027935367679</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>178</v>
       </c>
@@ -3754,11 +3788,11 @@
       <c r="F52" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G52" s="3">
-        <v>0.20996285574217635</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7">
+      <c r="G52" s="4">
+        <v>20.996285574217634</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>182</v>
       </c>
@@ -3777,11 +3811,11 @@
       <c r="F53" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G53" s="3">
-        <v>2.4268307705291758E-2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7">
+      <c r="G53" s="4">
+        <v>2.4268307705291758</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>186</v>
       </c>
@@ -3800,38 +3834,40 @@
       <c r="F54" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="G54" s="3">
-        <v>0.35000000000000014</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7">
+      <c r="G54" s="4">
+        <v>35.000000000000014</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
-      <c r="G55" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7">
+      <c r="G55" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
       <c r="D56" s="1"/>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
-    </row>
-    <row r="57" spans="1:7">
+      <c r="G56" s="4"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
       <c r="D57" s="1"/>
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
-    </row>
-    <row r="58" spans="1:7">
+      <c r="G57" s="4"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>190</v>
       </c>
@@ -3850,11 +3886,11 @@
       <c r="F58" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="G58" s="3">
-        <v>0.2730604585872386</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7">
+      <c r="G58" s="4">
+        <v>27.306045858723859</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>196</v>
       </c>
@@ -3873,11 +3909,11 @@
       <c r="F59" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="G59" s="3">
-        <v>0.27082277517680037</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7">
+      <c r="G59" s="4">
+        <v>27.082277517680037</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>200</v>
       </c>
@@ -3896,11 +3932,11 @@
       <c r="F60" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="G60" s="3">
-        <v>0.10611676623596111</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7">
+      <c r="G60" s="4">
+        <v>10.611676623596111</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>204</v>
       </c>
@@ -3919,38 +3955,40 @@
       <c r="F61" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="G61" s="3">
-        <v>0.34999999999999987</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7">
+      <c r="G61" s="4">
+        <v>34.999999999999986</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
-      <c r="G62" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7">
+      <c r="G62" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
-    </row>
-    <row r="64" spans="1:7">
+      <c r="G63" s="4"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
-    </row>
-    <row r="65" spans="1:7">
+      <c r="G64" s="4"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>208</v>
       </c>
@@ -3969,11 +4007,11 @@
       <c r="F65" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="G65" s="3">
-        <v>0.35000000000000059</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7">
+      <c r="G65" s="4">
+        <v>35.000000000000057</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>214</v>
       </c>
@@ -3992,11 +4030,11 @@
       <c r="F66" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="G66" s="3">
-        <v>0.3499999999999997</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7">
+      <c r="G66" s="4">
+        <v>34.999999999999972</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>218</v>
       </c>
@@ -4015,38 +4053,40 @@
       <c r="F67" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="G67" s="3">
-        <v>0.29999999999999977</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7">
+      <c r="G67" s="4">
+        <v>29.999999999999975</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
       <c r="D68" s="1"/>
       <c r="E68" s="1"/>
       <c r="F68" s="1"/>
-      <c r="G68" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7">
+      <c r="G68" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
       <c r="E69" s="1"/>
       <c r="F69" s="1"/>
-    </row>
-    <row r="70" spans="1:7">
+      <c r="G69" s="4"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
       <c r="D70" s="1"/>
       <c r="E70" s="1"/>
       <c r="F70" s="1"/>
-    </row>
-    <row r="71" spans="1:7">
+      <c r="G70" s="4"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>222</v>
       </c>
@@ -4065,11 +4105,11 @@
       <c r="F71" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G71" s="3">
-        <v>6.4268409414856755E-3</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7">
+      <c r="G71" s="4">
+        <v>0.64268409414856753</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>228</v>
       </c>
@@ -4088,11 +4128,11 @@
       <c r="F72" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G72" s="3">
-        <v>7.5609632256846875E-3</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7">
+      <c r="G72" s="4">
+        <v>0.7560963225684687</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>232</v>
       </c>
@@ -4111,11 +4151,11 @@
       <c r="F73" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G73" s="3">
-        <v>0.10730964996511956</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7">
+      <c r="G73" s="4">
+        <v>10.730964996511956</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>236</v>
       </c>
@@ -4134,11 +4174,11 @@
       <c r="F74" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G74" s="3">
-        <v>1.8195381853919022E-2</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7">
+      <c r="G74" s="4">
+        <v>1.8195381853919022</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>240</v>
       </c>
@@ -4157,11 +4197,11 @@
       <c r="F75" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G75" s="3">
-        <v>2.8763230310705963E-3</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7">
+      <c r="G75" s="4">
+        <v>0.28763230310705962</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>244</v>
       </c>
@@ -4180,11 +4220,11 @@
       <c r="F76" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G76" s="3">
-        <v>1.1884277463650641E-2</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7">
+      <c r="G76" s="4">
+        <v>1.1884277463650641</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>248</v>
       </c>
@@ -4203,11 +4243,11 @@
       <c r="F77" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G77" s="3">
-        <v>1.1619504571713266E-2</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7">
+      <c r="G77" s="4">
+        <v>1.1619504571713266</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>252</v>
       </c>
@@ -4226,11 +4266,11 @@
       <c r="F78" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G78" s="3">
-        <v>2.0183584913928219E-2</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7">
+      <c r="G78" s="4">
+        <v>2.0183584913928221</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>256</v>
       </c>
@@ -4249,11 +4289,11 @@
       <c r="F79" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G79" s="3">
-        <v>1.6906981841891464E-2</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7">
+      <c r="G79" s="4">
+        <v>1.6906981841891464</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>260</v>
       </c>
@@ -4272,11 +4312,11 @@
       <c r="F80" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G80" s="3">
-        <v>4.0438407763013712E-3</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7">
+      <c r="G80" s="4">
+        <v>0.40438407763013712</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>264</v>
       </c>
@@ -4295,11 +4335,11 @@
       <c r="F81" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G81" s="3">
-        <v>1.5405813605353192E-2</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7">
+      <c r="G81" s="4">
+        <v>1.5405813605353191</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>268</v>
       </c>
@@ -4318,11 +4358,11 @@
       <c r="F82" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G82" s="3">
-        <v>6.6797793859036426E-3</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7">
+      <c r="G82" s="4">
+        <v>0.66797793859036425</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>272</v>
       </c>
@@ -4341,11 +4381,11 @@
       <c r="F83" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G83" s="3">
-        <v>3.8358207836844873E-3</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7">
+      <c r="G83" s="4">
+        <v>0.38358207836844871</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>276</v>
       </c>
@@ -4364,11 +4404,11 @@
       <c r="F84" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G84" s="3">
-        <v>3.4247978584992125E-3</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7">
+      <c r="G84" s="4">
+        <v>0.34247978584992123</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>280</v>
       </c>
@@ -4387,11 +4427,11 @@
       <c r="F85" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G85" s="3">
-        <v>2.5241635747024743E-3</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7">
+      <c r="G85" s="4">
+        <v>0.25241635747024743</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>284</v>
       </c>
@@ -4410,11 +4450,11 @@
       <c r="F86" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G86" s="3">
-        <v>1.2863594472238192E-2</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7">
+      <c r="G86" s="4">
+        <v>1.2863594472238191</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>288</v>
       </c>
@@ -4433,11 +4473,11 @@
       <c r="F87" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G87" s="3">
-        <v>8.9446708811558237E-3</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7">
+      <c r="G87" s="4">
+        <v>0.8944670881155824</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>292</v>
       </c>
@@ -4456,11 +4496,11 @@
       <c r="F88" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G88" s="3">
-        <v>4.9193886569588192E-3</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7">
+      <c r="G88" s="4">
+        <v>0.49193886569588191</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>296</v>
       </c>
@@ -4479,11 +4519,11 @@
       <c r="F89" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G89" s="3">
-        <v>9.2233806084325923E-3</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7">
+      <c r="G89" s="4">
+        <v>0.9223380608432592</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>300</v>
       </c>
@@ -4502,11 +4542,11 @@
       <c r="F90" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G90" s="3">
-        <v>0.21741061772724746</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7">
+      <c r="G90" s="4">
+        <v>21.741061772724745</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>304</v>
       </c>
@@ -4525,11 +4565,11 @@
       <c r="F91" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G91" s="3">
-        <v>0.10039949438683722</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7">
+      <c r="G91" s="4">
+        <v>10.039949438683722</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>308</v>
       </c>
@@ -4548,11 +4588,11 @@
       <c r="F92" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G92" s="3">
-        <v>4.2991198253573171E-2</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7">
+      <c r="G92" s="4">
+        <v>4.2991198253573168</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>312</v>
       </c>
@@ -4571,11 +4611,11 @@
       <c r="F93" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G93" s="3">
-        <v>0.35000000000000009</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7">
+      <c r="G93" s="4">
+        <v>35.000000000000007</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>316</v>
       </c>
@@ -4594,11 +4634,11 @@
       <c r="F94" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G94" s="3">
-        <v>1.0912976642196931E-2</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7">
+      <c r="G94" s="4">
+        <v>1.091297664219693</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>320</v>
       </c>
@@ -4617,38 +4657,40 @@
       <c r="F95" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G95" s="3">
-        <v>3.4569545784522405E-3</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7">
+      <c r="G95" s="4">
+        <v>0.34569545784522404</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
       <c r="D96" s="1"/>
       <c r="E96" s="1"/>
       <c r="F96" s="1"/>
-      <c r="G96" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7">
+      <c r="G96" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
       <c r="D97" s="1"/>
       <c r="E97" s="1"/>
       <c r="F97" s="1"/>
-    </row>
-    <row r="98" spans="1:7">
+      <c r="G97" s="4"/>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
       <c r="D98" s="1"/>
       <c r="E98" s="1"/>
       <c r="F98" s="1"/>
-    </row>
-    <row r="99" spans="1:7">
+      <c r="G98" s="4"/>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>324</v>
       </c>
@@ -4667,11 +4709,11 @@
       <c r="F99" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G99" s="3">
-        <v>0.14534720742314677</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7">
+      <c r="G99" s="4">
+        <v>14.534720742314677</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>330</v>
       </c>
@@ -4690,11 +4732,11 @@
       <c r="F100" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G100" s="3">
-        <v>3.28718651985749E-2</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7">
+      <c r="G100" s="4">
+        <v>3.2871865198574901</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>334</v>
       </c>
@@ -4713,11 +4755,11 @@
       <c r="F101" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G101" s="3">
-        <v>1.2633066557741102E-2</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7">
+      <c r="G101" s="4">
+        <v>1.2633066557741102</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>338</v>
       </c>
@@ -4736,11 +4778,11 @@
       <c r="F102" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G102" s="3">
-        <v>0.1168530872083297</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7">
+      <c r="G102" s="4">
+        <v>11.685308720832969</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>342</v>
       </c>
@@ -4759,11 +4801,11 @@
       <c r="F103" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G103" s="3">
-        <v>7.4360338790014861E-3</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7">
+      <c r="G103" s="4">
+        <v>0.74360338790014857</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>346</v>
       </c>
@@ -4782,11 +4824,11 @@
       <c r="F104" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G104" s="3">
-        <v>1.8861819786645476E-2</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7">
+      <c r="G104" s="4">
+        <v>1.8861819786645477</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>350</v>
       </c>
@@ -4805,11 +4847,11 @@
       <c r="F105" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G105" s="3">
-        <v>9.3574613617230976E-2</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7">
+      <c r="G105" s="4">
+        <v>9.3574613617230984</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>354</v>
       </c>
@@ -4828,11 +4870,11 @@
       <c r="F106" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G106" s="3">
-        <v>2.6737544742955959E-2</v>
-      </c>
-    </row>
-    <row r="107" spans="1:7">
+      <c r="G106" s="4">
+        <v>2.6737544742955959</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>358</v>
       </c>
@@ -4851,11 +4893,11 @@
       <c r="F107" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G107" s="3">
-        <v>6.0162994533910018E-2</v>
-      </c>
-    </row>
-    <row r="108" spans="1:7">
+      <c r="G107" s="4">
+        <v>6.0162994533910021</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>362</v>
       </c>
@@ -4874,11 +4916,11 @@
       <c r="F108" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G108" s="3">
-        <v>2.3144064644394571E-2</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7">
+      <c r="G108" s="4">
+        <v>2.3144064644394571</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>366</v>
       </c>
@@ -4897,11 +4939,11 @@
       <c r="F109" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G109" s="3">
-        <v>1.1140049555567253E-2</v>
-      </c>
-    </row>
-    <row r="110" spans="1:7">
+      <c r="G109" s="4">
+        <v>1.1140049555567253</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>370</v>
       </c>
@@ -4920,11 +4962,11 @@
       <c r="F110" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G110" s="3">
-        <v>0.16699279568276421</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7">
+      <c r="G110" s="4">
+        <v>16.69927956827642</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>374</v>
       </c>
@@ -4943,11 +4985,11 @@
       <c r="F111" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G111" s="3">
-        <v>7.799032110121451E-2</v>
-      </c>
-    </row>
-    <row r="112" spans="1:7">
+      <c r="G111" s="4">
+        <v>7.799032110121451</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>378</v>
       </c>
@@ -4966,11 +5008,11 @@
       <c r="F112" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G112" s="3">
-        <v>0.1759654938084107</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7">
+      <c r="G112" s="4">
+        <v>17.596549380841068</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>382</v>
       </c>
@@ -4989,38 +5031,40 @@
       <c r="F113" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="G113" s="3">
-        <v>3.0289042260112319E-2</v>
-      </c>
-    </row>
-    <row r="114" spans="1:7">
+      <c r="G113" s="4">
+        <v>3.0289042260112318</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
       <c r="D114" s="1"/>
       <c r="E114" s="1"/>
       <c r="F114" s="1"/>
-      <c r="G114" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7">
+      <c r="G114" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
       <c r="D115" s="1"/>
       <c r="E115" s="1"/>
       <c r="F115" s="1"/>
-    </row>
-    <row r="116" spans="1:7">
+      <c r="G115" s="4"/>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
       <c r="D116" s="1"/>
       <c r="E116" s="1"/>
       <c r="F116" s="1"/>
-    </row>
-    <row r="117" spans="1:7">
+      <c r="G116" s="4"/>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>386</v>
       </c>
@@ -5039,11 +5083,11 @@
       <c r="F117" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="G117" s="3">
-        <v>5.0095362938591521E-2</v>
-      </c>
-    </row>
-    <row r="118" spans="1:7">
+      <c r="G117" s="4">
+        <v>5.0095362938591519</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>392</v>
       </c>
@@ -5062,11 +5106,11 @@
       <c r="F118" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="G118" s="3">
-        <v>0.35000000000000009</v>
-      </c>
-    </row>
-    <row r="119" spans="1:7">
+      <c r="G118" s="4">
+        <v>35.000000000000007</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>396</v>
       </c>
@@ -5085,11 +5129,11 @@
       <c r="F119" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="G119" s="3">
-        <v>3.0110698603456172E-2</v>
-      </c>
-    </row>
-    <row r="120" spans="1:7">
+      <c r="G119" s="4">
+        <v>3.0110698603456174</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>400</v>
       </c>
@@ -5108,11 +5152,11 @@
       <c r="F120" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="G120" s="3">
-        <v>3.7954486278303358E-3</v>
-      </c>
-    </row>
-    <row r="121" spans="1:7">
+      <c r="G120" s="4">
+        <v>0.37954486278303357</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>404</v>
       </c>
@@ -5131,11 +5175,11 @@
       <c r="F121" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="G121" s="3">
-        <v>0.24908986560673474</v>
-      </c>
-    </row>
-    <row r="122" spans="1:7">
+      <c r="G121" s="4">
+        <v>24.908986560673473</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>408</v>
       </c>
@@ -5154,11 +5198,11 @@
       <c r="F122" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="G122" s="3">
-        <v>0.29885427516436724</v>
-      </c>
-    </row>
-    <row r="123" spans="1:7">
+      <c r="G122" s="4">
+        <v>29.885427516436724</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>412</v>
       </c>
@@ -5177,38 +5221,40 @@
       <c r="F123" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="G123" s="3">
-        <v>1.8054349059020036E-2</v>
-      </c>
-    </row>
-    <row r="124" spans="1:7">
+      <c r="G123" s="4">
+        <v>1.8054349059020036</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
       <c r="C124" s="1"/>
       <c r="D124" s="1"/>
       <c r="E124" s="1"/>
       <c r="F124" s="1"/>
-      <c r="G124" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="125" spans="1:7">
+      <c r="G124" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
       <c r="C125" s="1"/>
       <c r="D125" s="1"/>
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
-    </row>
-    <row r="126" spans="1:7">
+      <c r="G125" s="4"/>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
       <c r="C126" s="1"/>
       <c r="D126" s="1"/>
       <c r="E126" s="1"/>
       <c r="F126" s="1"/>
-    </row>
-    <row r="127" spans="1:7">
+      <c r="G126" s="4"/>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>416</v>
       </c>
@@ -5227,11 +5273,11 @@
       <c r="F127" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="G127" s="3">
-        <v>1.6354383307310781E-2</v>
-      </c>
-    </row>
-    <row r="128" spans="1:7">
+      <c r="G127" s="4">
+        <v>1.635438330731078</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>422</v>
       </c>
@@ -5250,11 +5296,11 @@
       <c r="F128" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="G128" s="3">
-        <v>2.8363525608471676E-2</v>
-      </c>
-    </row>
-    <row r="129" spans="1:7">
+      <c r="G128" s="4">
+        <v>2.8363525608471676</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>426</v>
       </c>
@@ -5273,11 +5319,11 @@
       <c r="F129" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="G129" s="3">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="130" spans="1:7">
+      <c r="G129" s="4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>430</v>
       </c>
@@ -5296,11 +5342,11 @@
       <c r="F130" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="G130" s="3">
-        <v>2.4782967011310053E-2</v>
-      </c>
-    </row>
-    <row r="131" spans="1:7">
+      <c r="G130" s="4">
+        <v>2.4782967011310051</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>434</v>
       </c>
@@ -5319,11 +5365,11 @@
       <c r="F131" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="G131" s="3">
-        <v>0.1133331204683236</v>
-      </c>
-    </row>
-    <row r="132" spans="1:7">
+      <c r="G131" s="4">
+        <v>11.33331204683236</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>438</v>
       </c>
@@ -5342,11 +5388,11 @@
       <c r="F132" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="G132" s="3">
-        <v>0.11716600360458408</v>
-      </c>
-    </row>
-    <row r="133" spans="1:7">
+      <c r="G132" s="4">
+        <v>11.716600360458408</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>442</v>
       </c>
@@ -5365,38 +5411,40 @@
       <c r="F133" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="G133" s="3">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="134" spans="1:7">
+      <c r="G133" s="4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
       <c r="C134" s="1"/>
       <c r="D134" s="1"/>
       <c r="E134" s="1"/>
       <c r="F134" s="1"/>
-      <c r="G134" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="135" spans="1:7">
+      <c r="G134" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
       <c r="C135" s="1"/>
       <c r="D135" s="1"/>
       <c r="E135" s="1"/>
       <c r="F135" s="1"/>
-    </row>
-    <row r="136" spans="1:7">
+      <c r="G135" s="4"/>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
       <c r="C136" s="1"/>
       <c r="D136" s="1"/>
       <c r="E136" s="1"/>
       <c r="F136" s="1"/>
-    </row>
-    <row r="137" spans="1:7">
+      <c r="G136" s="4"/>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>446</v>
       </c>
@@ -5415,11 +5463,11 @@
       <c r="F137" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G137" s="3">
-        <v>6.1723640322048166E-3</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7">
+      <c r="G137" s="4">
+        <v>0.61723640322048168</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>452</v>
       </c>
@@ -5438,11 +5486,11 @@
       <c r="F138" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G138" s="3">
-        <v>6.069638286180886E-2</v>
-      </c>
-    </row>
-    <row r="139" spans="1:7">
+      <c r="G138" s="4">
+        <v>6.0696382861808864</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>456</v>
       </c>
@@ -5461,11 +5509,11 @@
       <c r="F139" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G139" s="3">
-        <v>1.4941712547963381E-2</v>
-      </c>
-    </row>
-    <row r="140" spans="1:7">
+      <c r="G139" s="4">
+        <v>1.4941712547963382</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>460</v>
       </c>
@@ -5484,11 +5532,11 @@
       <c r="F140" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G140" s="3">
-        <v>5.1210729325992079E-3</v>
-      </c>
-    </row>
-    <row r="141" spans="1:7">
+      <c r="G140" s="4">
+        <v>0.51210729325992077</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>464</v>
       </c>
@@ -5507,11 +5555,11 @@
       <c r="F141" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G141" s="3">
-        <v>8.7782661407787628E-4</v>
-      </c>
-    </row>
-    <row r="142" spans="1:7">
+      <c r="G141" s="4">
+        <v>8.7782661407787635E-2</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>468</v>
       </c>
@@ -5530,11 +5578,11 @@
       <c r="F142" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G142" s="3">
-        <v>1.6317990605618326E-4</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7">
+      <c r="G142" s="4">
+        <v>1.6317990605618327E-2</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>472</v>
       </c>
@@ -5553,11 +5601,11 @@
       <c r="F143" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G143" s="3">
-        <v>3.4987588482255504E-3</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7">
+      <c r="G143" s="4">
+        <v>0.34987588482255505</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>476</v>
       </c>
@@ -5576,11 +5624,11 @@
       <c r="F144" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G144" s="3">
-        <v>1.5512299627493106E-2</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7">
+      <c r="G144" s="4">
+        <v>1.5512299627493107</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>480</v>
       </c>
@@ -5599,11 +5647,11 @@
       <c r="F145" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G145" s="3">
-        <v>4.8293423157115501E-3</v>
-      </c>
-    </row>
-    <row r="146" spans="1:7">
+      <c r="G145" s="4">
+        <v>0.482934231571155</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>484</v>
       </c>
@@ -5622,11 +5670,11 @@
       <c r="F146" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G146" s="3">
-        <v>2.1090059554873578E-3</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7">
+      <c r="G146" s="4">
+        <v>0.21090059554873578</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>488</v>
       </c>
@@ -5645,11 +5693,11 @@
       <c r="F147" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G147" s="3">
-        <v>1.7421801721905486E-3</v>
-      </c>
-    </row>
-    <row r="148" spans="1:7">
+      <c r="G147" s="4">
+        <v>0.17421801721905486</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>492</v>
       </c>
@@ -5668,11 +5716,11 @@
       <c r="F148" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G148" s="3">
-        <v>4.5375189444402664E-2</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7">
+      <c r="G148" s="4">
+        <v>4.5375189444402668</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>496</v>
       </c>
@@ -5691,11 +5739,11 @@
       <c r="F149" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G149" s="3">
-        <v>0.12493639892769719</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7">
+      <c r="G149" s="4">
+        <v>12.493639892769719</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>500</v>
       </c>
@@ -5714,11 +5762,11 @@
       <c r="F150" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G150" s="3">
-        <v>5.8825118996496492E-2</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7">
+      <c r="G150" s="4">
+        <v>5.882511899649649</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>504</v>
       </c>
@@ -5737,11 +5785,11 @@
       <c r="F151" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G151" s="3">
-        <v>0.22880164906768613</v>
-      </c>
-    </row>
-    <row r="152" spans="1:7">
+      <c r="G151" s="4">
+        <v>22.880164906768613</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>508</v>
       </c>
@@ -5760,11 +5808,11 @@
       <c r="F152" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G152" s="3">
-        <v>1.4662439100680019E-2</v>
-      </c>
-    </row>
-    <row r="153" spans="1:7">
+      <c r="G152" s="4">
+        <v>1.4662439100680018</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>512</v>
       </c>
@@ -5783,11 +5831,11 @@
       <c r="F153" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G153" s="3">
-        <v>7.6848589158820335E-3</v>
-      </c>
-    </row>
-    <row r="154" spans="1:7">
+      <c r="G153" s="4">
+        <v>0.76848589158820335</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>516</v>
       </c>
@@ -5806,11 +5854,11 @@
       <c r="F154" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G154" s="3">
-        <v>0.10903079513674047</v>
-      </c>
-    </row>
-    <row r="155" spans="1:7">
+      <c r="G154" s="4">
+        <v>10.903079513674047</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>520</v>
       </c>
@@ -5829,11 +5877,11 @@
       <c r="F155" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G155" s="3">
-        <v>1.0207405572770752E-2</v>
-      </c>
-    </row>
-    <row r="156" spans="1:7">
+      <c r="G155" s="4">
+        <v>1.0207405572770751</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>524</v>
       </c>
@@ -5852,11 +5900,11 @@
       <c r="F156" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G156" s="3">
-        <v>6.8914910184001157E-2</v>
-      </c>
-    </row>
-    <row r="157" spans="1:7">
+      <c r="G156" s="4">
+        <v>6.8914910184001155</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>528</v>
       </c>
@@ -5875,11 +5923,11 @@
       <c r="F157" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G157" s="3">
-        <v>4.8103001362130113E-3</v>
-      </c>
-    </row>
-    <row r="158" spans="1:7">
+      <c r="G157" s="4">
+        <v>0.48103001362130116</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>532</v>
       </c>
@@ -5898,11 +5946,11 @@
       <c r="F158" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G158" s="3">
-        <v>1.4363623434841797E-2</v>
-      </c>
-    </row>
-    <row r="159" spans="1:7">
+      <c r="G158" s="4">
+        <v>1.4363623434841797</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>536</v>
       </c>
@@ -5921,11 +5969,11 @@
       <c r="F159" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G159" s="3">
-        <v>1.2361380533054503E-2</v>
-      </c>
-    </row>
-    <row r="160" spans="1:7">
+      <c r="G159" s="4">
+        <v>1.2361380533054502</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>540</v>
       </c>
@@ -5944,11 +5992,11 @@
       <c r="F160" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G160" s="3">
-        <v>0.15295530429924467</v>
-      </c>
-    </row>
-    <row r="161" spans="1:7">
+      <c r="G160" s="4">
+        <v>15.295530429924467</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>544</v>
       </c>
@@ -5967,11 +6015,11 @@
       <c r="F161" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G161" s="3">
-        <v>1.4279581972368199E-2</v>
-      </c>
-    </row>
-    <row r="162" spans="1:7">
+      <c r="G161" s="4">
+        <v>1.42795819723682</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>548</v>
       </c>
@@ -5990,38 +6038,40 @@
       <c r="F162" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="G162" s="3">
-        <v>1.712691846410256E-2</v>
-      </c>
-    </row>
-    <row r="163" spans="1:7">
+      <c r="G162" s="4">
+        <v>1.7126918464102561</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="1"/>
       <c r="B163" s="1"/>
       <c r="C163" s="1"/>
       <c r="D163" s="1"/>
       <c r="E163" s="1"/>
       <c r="F163" s="1"/>
-      <c r="G163" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="164" spans="1:7">
+      <c r="G163" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="1"/>
       <c r="B164" s="1"/>
       <c r="C164" s="1"/>
       <c r="D164" s="1"/>
       <c r="E164" s="1"/>
       <c r="F164" s="1"/>
-    </row>
-    <row r="165" spans="1:7">
+      <c r="G164" s="4"/>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" s="1"/>
       <c r="B165" s="1"/>
       <c r="C165" s="1"/>
       <c r="D165" s="1"/>
       <c r="E165" s="1"/>
       <c r="F165" s="1"/>
-    </row>
-    <row r="166" spans="1:7">
+      <c r="G165" s="4"/>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
         <v>552</v>
       </c>
@@ -6040,11 +6090,11 @@
       <c r="F166" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G166" s="3">
-        <v>9.9657725191690267E-3</v>
-      </c>
-    </row>
-    <row r="167" spans="1:7">
+      <c r="G166" s="4">
+        <v>0.99657725191690272</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>558</v>
       </c>
@@ -6063,11 +6113,11 @@
       <c r="F167" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G167" s="3">
-        <v>3.6362145086495525E-2</v>
-      </c>
-    </row>
-    <row r="168" spans="1:7">
+      <c r="G167" s="4">
+        <v>3.6362145086495525</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>562</v>
       </c>
@@ -6086,11 +6136,11 @@
       <c r="F168" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G168" s="3">
-        <v>2.9949343378586511E-3</v>
-      </c>
-    </row>
-    <row r="169" spans="1:7">
+      <c r="G168" s="4">
+        <v>0.29949343378586513</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>566</v>
       </c>
@@ -6109,11 +6159,11 @@
       <c r="F169" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G169" s="3">
-        <v>5.1132228634460956E-3</v>
-      </c>
-    </row>
-    <row r="170" spans="1:7">
+      <c r="G169" s="4">
+        <v>0.51132228634460952</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>570</v>
       </c>
@@ -6132,11 +6182,11 @@
       <c r="F170" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G170" s="3">
-        <v>2.2772456615385473E-3</v>
-      </c>
-    </row>
-    <row r="171" spans="1:7">
+      <c r="G170" s="4">
+        <v>0.22772456615385472</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>574</v>
       </c>
@@ -6155,11 +6205,11 @@
       <c r="F171" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G171" s="3">
-        <v>3.0343958240828781E-2</v>
-      </c>
-    </row>
-    <row r="172" spans="1:7">
+      <c r="G171" s="4">
+        <v>3.0343958240828783</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
         <v>578</v>
       </c>
@@ -6178,11 +6228,11 @@
       <c r="F172" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G172" s="3">
-        <v>7.9044930632569503E-3</v>
-      </c>
-    </row>
-    <row r="173" spans="1:7">
+      <c r="G172" s="4">
+        <v>0.79044930632569499</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
         <v>582</v>
       </c>
@@ -6201,11 +6251,11 @@
       <c r="F173" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G173" s="3">
-        <v>6.7243161131449103E-3</v>
-      </c>
-    </row>
-    <row r="174" spans="1:7">
+      <c r="G173" s="4">
+        <v>0.67243161131449103</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>586</v>
       </c>
@@ -6224,11 +6274,11 @@
       <c r="F174" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G174" s="3">
-        <v>1.0342542064508778E-2</v>
-      </c>
-    </row>
-    <row r="175" spans="1:7">
+      <c r="G174" s="4">
+        <v>1.0342542064508777</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>590</v>
       </c>
@@ -6247,11 +6297,11 @@
       <c r="F175" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G175" s="3">
-        <v>9.3821617503280844E-3</v>
-      </c>
-    </row>
-    <row r="176" spans="1:7">
+      <c r="G175" s="4">
+        <v>0.93821617503280841</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
         <v>594</v>
       </c>
@@ -6270,11 +6320,11 @@
       <c r="F176" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G176" s="3">
-        <v>2.1053583907871031E-3</v>
-      </c>
-    </row>
-    <row r="177" spans="1:7">
+      <c r="G176" s="4">
+        <v>0.21053583907871032</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
         <v>598</v>
       </c>
@@ -6293,11 +6343,11 @@
       <c r="F177" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G177" s="3">
-        <v>8.0518436747952244E-3</v>
-      </c>
-    </row>
-    <row r="178" spans="1:7">
+      <c r="G177" s="4">
+        <v>0.80518436747952249</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
         <v>602</v>
       </c>
@@ -6316,11 +6366,11 @@
       <c r="F178" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G178" s="3">
-        <v>3.4183498466265334E-3</v>
-      </c>
-    </row>
-    <row r="179" spans="1:7">
+      <c r="G178" s="4">
+        <v>0.34183498466265333</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
         <v>606</v>
       </c>
@@ -6339,11 +6389,11 @@
       <c r="F179" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G179" s="3">
-        <v>2.6527246116734731E-3</v>
-      </c>
-    </row>
-    <row r="180" spans="1:7">
+      <c r="G179" s="4">
+        <v>0.26527246116734732</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
         <v>610</v>
       </c>
@@ -6362,11 +6412,11 @@
       <c r="F180" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G180" s="3">
-        <v>3.6844105687238813E-3</v>
-      </c>
-    </row>
-    <row r="181" spans="1:7">
+      <c r="G180" s="4">
+        <v>0.36844105687238815</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
         <v>614</v>
       </c>
@@ -6385,11 +6435,11 @@
       <c r="F181" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G181" s="3">
-        <v>6.6949136450885641E-2</v>
-      </c>
-    </row>
-    <row r="182" spans="1:7">
+      <c r="G181" s="4">
+        <v>6.6949136450885645</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
         <v>618</v>
       </c>
@@ -6408,11 +6458,11 @@
       <c r="F182" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G182" s="3">
-        <v>6.6818593107499311E-2</v>
-      </c>
-    </row>
-    <row r="183" spans="1:7">
+      <c r="G182" s="4">
+        <v>6.6818593107499309</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
         <v>622</v>
       </c>
@@ -6431,11 +6481,11 @@
       <c r="F183" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G183" s="3">
-        <v>0.10828204989201327</v>
-      </c>
-    </row>
-    <row r="184" spans="1:7">
+      <c r="G183" s="4">
+        <v>10.828204989201327</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
         <v>626</v>
       </c>
@@ -6454,11 +6504,11 @@
       <c r="F184" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G184" s="3">
-        <v>1.453671279506635E-2</v>
-      </c>
-    </row>
-    <row r="185" spans="1:7">
+      <c r="G184" s="4">
+        <v>1.4536712795066349</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
         <v>630</v>
       </c>
@@ -6477,11 +6527,11 @@
       <c r="F185" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G185" s="3">
-        <v>4.5297494838276442E-2</v>
-      </c>
-    </row>
-    <row r="186" spans="1:7">
+      <c r="G185" s="4">
+        <v>4.5297494838276444</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
         <v>634</v>
       </c>
@@ -6500,11 +6550,11 @@
       <c r="F186" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G186" s="3">
-        <v>8.3465817760985783E-3</v>
-      </c>
-    </row>
-    <row r="187" spans="1:7">
+      <c r="G186" s="4">
+        <v>0.83465817760985783</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
         <v>638</v>
       </c>
@@ -6523,11 +6573,11 @@
       <c r="F187" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G187" s="3">
-        <v>5.1650064349498127E-2</v>
-      </c>
-    </row>
-    <row r="188" spans="1:7">
+      <c r="G187" s="4">
+        <v>5.165006434949813</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
         <v>642</v>
       </c>
@@ -6546,11 +6596,11 @@
       <c r="F188" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G188" s="3">
-        <v>1.6137155547535201E-2</v>
-      </c>
-    </row>
-    <row r="189" spans="1:7">
+      <c r="G188" s="4">
+        <v>1.6137155547535202</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
         <v>646</v>
       </c>
@@ -6569,11 +6619,11 @@
       <c r="F189" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G189" s="3">
-        <v>3.5382363087503132E-3</v>
-      </c>
-    </row>
-    <row r="190" spans="1:7">
+      <c r="G189" s="4">
+        <v>0.35382363087503133</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
         <v>650</v>
       </c>
@@ -6592,11 +6642,11 @@
       <c r="F190" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G190" s="3">
-        <v>0.35000000000000009</v>
-      </c>
-    </row>
-    <row r="191" spans="1:7">
+      <c r="G190" s="4">
+        <v>35.000000000000007</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
         <v>654</v>
       </c>
@@ -6615,11 +6665,11 @@
       <c r="F191" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G191" s="3">
-        <v>2.3830653317919372E-2</v>
-      </c>
-    </row>
-    <row r="192" spans="1:7">
+      <c r="G191" s="4">
+        <v>2.3830653317919372</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
         <v>658</v>
       </c>
@@ -6638,11 +6688,11 @@
       <c r="F192" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G192" s="3">
-        <v>1.0088966583683261E-2</v>
-      </c>
-    </row>
-    <row r="193" spans="1:7">
+      <c r="G192" s="4">
+        <v>1.0088966583683261</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
         <v>662</v>
       </c>
@@ -6661,11 +6711,11 @@
       <c r="F193" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G193" s="3">
-        <v>9.0852065603730894E-2</v>
-      </c>
-    </row>
-    <row r="194" spans="1:7">
+      <c r="G193" s="4">
+        <v>9.0852065603730896</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>666</v>
       </c>
@@ -6684,38 +6734,40 @@
       <c r="F194" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="G194" s="3">
-        <v>2.3488106358615412E-3</v>
-      </c>
-    </row>
-    <row r="195" spans="1:7">
+      <c r="G194" s="4">
+        <v>0.23488106358615413</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" s="1"/>
       <c r="B195" s="1"/>
       <c r="C195" s="1"/>
       <c r="D195" s="1"/>
       <c r="E195" s="1"/>
       <c r="F195" s="1"/>
-      <c r="G195" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="196" spans="1:7">
+      <c r="G195" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" s="1"/>
       <c r="B196" s="1"/>
       <c r="C196" s="1"/>
       <c r="D196" s="1"/>
       <c r="E196" s="1"/>
       <c r="F196" s="1"/>
-    </row>
-    <row r="197" spans="1:7">
+      <c r="G196" s="4"/>
+    </row>
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" s="1"/>
       <c r="B197" s="1"/>
       <c r="C197" s="1"/>
       <c r="D197" s="1"/>
       <c r="E197" s="1"/>
       <c r="F197" s="1"/>
-    </row>
-    <row r="198" spans="1:7">
+      <c r="G197" s="4"/>
+    </row>
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
         <v>670</v>
       </c>
@@ -6734,11 +6786,11 @@
       <c r="F198" s="1" t="s">
         <v>675</v>
       </c>
-      <c r="G198" s="3">
-        <v>0.34999999999999987</v>
-      </c>
-    </row>
-    <row r="199" spans="1:7">
+      <c r="G198" s="4">
+        <v>34.999999999999986</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
         <v>676</v>
       </c>
@@ -6757,11 +6809,11 @@
       <c r="F199" s="1" t="s">
         <v>675</v>
       </c>
-      <c r="G199" s="3">
-        <v>0.35000000000000009</v>
-      </c>
-    </row>
-    <row r="200" spans="1:7">
+      <c r="G199" s="4">
+        <v>35.000000000000007</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
         <v>680</v>
       </c>
@@ -6780,38 +6832,40 @@
       <c r="F200" s="1" t="s">
         <v>675</v>
       </c>
-      <c r="G200" s="3">
-        <v>0.29999999999999993</v>
-      </c>
-    </row>
-    <row r="201" spans="1:7">
+      <c r="G200" s="4">
+        <v>29.999999999999993</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" s="1"/>
       <c r="B201" s="1"/>
       <c r="C201" s="1"/>
       <c r="D201" s="1"/>
       <c r="E201" s="1"/>
       <c r="F201" s="1"/>
-      <c r="G201" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="202" spans="1:7">
+      <c r="G201" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202" s="1"/>
       <c r="B202" s="1"/>
       <c r="C202" s="1"/>
       <c r="D202" s="1"/>
       <c r="E202" s="1"/>
       <c r="F202" s="1"/>
-    </row>
-    <row r="203" spans="1:7">
+      <c r="G202" s="4"/>
+    </row>
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203" s="1"/>
       <c r="B203" s="1"/>
       <c r="C203" s="1"/>
       <c r="D203" s="1"/>
       <c r="E203" s="1"/>
       <c r="F203" s="1"/>
-    </row>
-    <row r="204" spans="1:7">
+      <c r="G203" s="4"/>
+    </row>
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>684</v>
       </c>
@@ -6830,11 +6884,11 @@
       <c r="F204" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="G204" s="3">
-        <v>0.26170604673549436</v>
-      </c>
-    </row>
-    <row r="205" spans="1:7">
+      <c r="G204" s="4">
+        <v>26.170604673549434</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
         <v>690</v>
       </c>
@@ -6853,11 +6907,11 @@
       <c r="F205" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="G205" s="3">
-        <v>7.2641730622261397E-2</v>
-      </c>
-    </row>
-    <row r="206" spans="1:7">
+      <c r="G205" s="4">
+        <v>7.2641730622261393</v>
+      </c>
+    </row>
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
         <v>694</v>
       </c>
@@ -6876,11 +6930,11 @@
       <c r="F206" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="G206" s="3">
-        <v>0.10820610271628164</v>
-      </c>
-    </row>
-    <row r="207" spans="1:7">
+      <c r="G206" s="4">
+        <v>10.820610271628164</v>
+      </c>
+    </row>
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
         <v>698</v>
       </c>
@@ -6899,11 +6953,11 @@
       <c r="F207" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="G207" s="3">
-        <v>0.32539472749514797</v>
-      </c>
-    </row>
-    <row r="208" spans="1:7">
+      <c r="G207" s="4">
+        <v>32.5394727495148</v>
+      </c>
+    </row>
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
         <v>702</v>
       </c>
@@ -6922,11 +6976,11 @@
       <c r="F208" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="G208" s="3">
-        <v>0.1019278873140403</v>
-      </c>
-    </row>
-    <row r="209" spans="1:7">
+      <c r="G208" s="4">
+        <v>10.192788731404031</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
         <v>706</v>
       </c>
@@ -6945,11 +6999,11 @@
       <c r="F209" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="G209" s="3">
-        <v>0.10403302219915783</v>
-      </c>
-    </row>
-    <row r="210" spans="1:7">
+      <c r="G209" s="4">
+        <v>10.403302219915783</v>
+      </c>
+    </row>
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
         <v>710</v>
       </c>
@@ -6968,11 +7022,11 @@
       <c r="F210" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="G210" s="3">
-        <v>6.8489468341638585E-3</v>
-      </c>
-    </row>
-    <row r="211" spans="1:7">
+      <c r="G210" s="4">
+        <v>0.68489468341638582</v>
+      </c>
+    </row>
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
         <v>714</v>
       </c>
@@ -6991,38 +7045,40 @@
       <c r="F211" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="G211" s="3">
-        <v>1.9241536083452467E-2</v>
-      </c>
-    </row>
-    <row r="212" spans="1:7">
+      <c r="G211" s="4">
+        <v>1.9241536083452466</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A212" s="1"/>
       <c r="B212" s="1"/>
       <c r="C212" s="1"/>
       <c r="D212" s="1"/>
       <c r="E212" s="1"/>
       <c r="F212" s="1"/>
-      <c r="G212" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="213" spans="1:7">
+      <c r="G212" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A213" s="1"/>
       <c r="B213" s="1"/>
       <c r="C213" s="1"/>
       <c r="D213" s="1"/>
       <c r="E213" s="1"/>
       <c r="F213" s="1"/>
-    </row>
-    <row r="214" spans="1:7">
+      <c r="G213" s="4"/>
+    </row>
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" s="1"/>
       <c r="B214" s="1"/>
       <c r="C214" s="1"/>
       <c r="D214" s="1"/>
       <c r="E214" s="1"/>
       <c r="F214" s="1"/>
-    </row>
-    <row r="215" spans="1:7">
+      <c r="G214" s="4"/>
+    </row>
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
         <v>718</v>
       </c>
@@ -7041,11 +7097,11 @@
       <c r="F215" s="1" t="s">
         <v>723</v>
       </c>
-      <c r="G215" s="3">
-        <v>0.24037524364633664</v>
-      </c>
-    </row>
-    <row r="216" spans="1:7">
+      <c r="G215" s="4">
+        <v>24.037524364633665</v>
+      </c>
+    </row>
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
         <v>724</v>
       </c>
@@ -7064,11 +7120,11 @@
       <c r="F216" s="1" t="s">
         <v>723</v>
       </c>
-      <c r="G216" s="3">
-        <v>3.5834246120822942E-2</v>
-      </c>
-    </row>
-    <row r="217" spans="1:7">
+      <c r="G216" s="4">
+        <v>3.5834246120822941</v>
+      </c>
+    </row>
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
         <v>728</v>
       </c>
@@ -7087,11 +7143,11 @@
       <c r="F217" s="1" t="s">
         <v>723</v>
       </c>
-      <c r="G217" s="3">
-        <v>8.3449741004382613E-2</v>
-      </c>
-    </row>
-    <row r="218" spans="1:7">
+      <c r="G217" s="4">
+        <v>8.3449741004382609</v>
+      </c>
+    </row>
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
         <v>732</v>
       </c>
@@ -7110,11 +7166,11 @@
       <c r="F218" s="1" t="s">
         <v>723</v>
       </c>
-      <c r="G218" s="3">
-        <v>0.11343363803257897</v>
-      </c>
-    </row>
-    <row r="219" spans="1:7">
+      <c r="G218" s="4">
+        <v>11.343363803257898</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
         <v>736</v>
       </c>
@@ -7133,11 +7189,11 @@
       <c r="F219" s="1" t="s">
         <v>723</v>
       </c>
-      <c r="G219" s="3">
-        <v>0.26785223873577324</v>
-      </c>
-    </row>
-    <row r="220" spans="1:7">
+      <c r="G219" s="4">
+        <v>26.785223873577323</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
         <v>740</v>
       </c>
@@ -7156,38 +7212,40 @@
       <c r="F220" s="1" t="s">
         <v>723</v>
       </c>
-      <c r="G220" s="3">
-        <v>0.25905489246010555</v>
-      </c>
-    </row>
-    <row r="221" spans="1:7">
+      <c r="G220" s="4">
+        <v>25.905489246010553</v>
+      </c>
+    </row>
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" s="1"/>
       <c r="B221" s="1"/>
       <c r="C221" s="1"/>
       <c r="D221" s="1"/>
       <c r="E221" s="1"/>
       <c r="F221" s="1"/>
-      <c r="G221" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="222" spans="1:7">
+      <c r="G221" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" s="1"/>
       <c r="B222" s="1"/>
       <c r="C222" s="1"/>
       <c r="D222" s="1"/>
       <c r="E222" s="1"/>
       <c r="F222" s="1"/>
-    </row>
-    <row r="223" spans="1:7">
+      <c r="G222" s="4"/>
+    </row>
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223" s="1"/>
       <c r="B223" s="1"/>
       <c r="C223" s="1"/>
       <c r="D223" s="1"/>
       <c r="E223" s="1"/>
       <c r="F223" s="1"/>
-    </row>
-    <row r="224" spans="1:7">
+      <c r="G223" s="4"/>
+    </row>
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
         <v>744</v>
       </c>
@@ -7206,11 +7264,11 @@
       <c r="F224" s="1" t="s">
         <v>749</v>
       </c>
-      <c r="G224" s="3">
-        <v>0.17712914313142364</v>
-      </c>
-    </row>
-    <row r="225" spans="1:7">
+      <c r="G224" s="4">
+        <v>17.712914313142363</v>
+      </c>
+    </row>
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225" s="1" t="s">
         <v>750</v>
       </c>
@@ -7229,11 +7287,11 @@
       <c r="F225" s="1" t="s">
         <v>749</v>
       </c>
-      <c r="G225" s="3">
-        <v>0.22672872483851181</v>
-      </c>
-    </row>
-    <row r="226" spans="1:7">
+      <c r="G225" s="4">
+        <v>22.672872483851179</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226" s="1" t="s">
         <v>754</v>
       </c>
@@ -7252,11 +7310,11 @@
       <c r="F226" s="1" t="s">
         <v>749</v>
       </c>
-      <c r="G226" s="3">
-        <v>0.34220183955766331</v>
-      </c>
-    </row>
-    <row r="227" spans="1:7">
+      <c r="G226" s="4">
+        <v>34.220183955766331</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
         <v>758</v>
       </c>
@@ -7275,11 +7333,11 @@
       <c r="F227" s="1" t="s">
         <v>749</v>
       </c>
-      <c r="G227" s="3">
-        <v>0.23332747478949209</v>
-      </c>
-    </row>
-    <row r="228" spans="1:7">
+      <c r="G227" s="4">
+        <v>23.332747478949209</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A228" s="1" t="s">
         <v>762</v>
       </c>
@@ -7298,13 +7356,13 @@
       <c r="F228" s="1" t="s">
         <v>749</v>
       </c>
-      <c r="G228" s="3">
-        <v>2.0612817682909124E-2</v>
-      </c>
-    </row>
-    <row r="229" spans="1:7">
-      <c r="G229" s="3">
-        <v>1</v>
+      <c r="G228" s="4">
+        <v>2.0612817682909124</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G229" s="4">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>